<commit_message>
Added teeset name to points worksheet
</commit_message>
<xml_diff>
--- a/templates/excel/MatchAid_PointScoring_2x9_Template.xlsx
+++ b/templates/excel/MatchAid_PointScoring_2x9_Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e0bc09bc27ca3c1c/Documents/GitHub/MatchAid_GoDaddy/templates/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="26" documentId="8_{60F95BE6-3508-4CA1-8C3C-FCCA8C8EEC95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1CA5815F-E87F-44D6-93F6-40F00684E940}"/>
+  <xr:revisionPtr revIDLastSave="43" documentId="8_{60F95BE6-3508-4CA1-8C3C-FCCA8C8EEC95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DAB6D47C-F73E-4769-AAA9-39841AB98039}"/>
   <bookViews>
-    <workbookView xWindow="-12" yWindow="0" windowWidth="16584" windowHeight="13704" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Group Template" sheetId="1" r:id="rId1"/>
@@ -31,15 +31,19 @@
     <definedName name="Table1_Player1_DisplayName" localSheetId="0">'Group Template'!$B$3</definedName>
     <definedName name="Table1_Player1_PairingPos" localSheetId="0">'Group Template'!$A$3</definedName>
     <definedName name="Table1_Player1_Quota" localSheetId="0">'Group Template'!$C$3</definedName>
+    <definedName name="Table1_Player1_TeeSetName" localSheetId="0">'Group Template'!$C$25</definedName>
     <definedName name="Table1_Player2_DisplayName" localSheetId="0">'Group Template'!$B$5</definedName>
     <definedName name="Table1_Player2_PairingPos" localSheetId="0">'Group Template'!$A$5</definedName>
     <definedName name="Table1_Player2_Quota" localSheetId="0">'Group Template'!$C$5</definedName>
+    <definedName name="Table1_Player2_TeeSetName" localSheetId="0">'Group Template'!$C$26</definedName>
     <definedName name="Table1_Player3_DisplayName" localSheetId="0">'Group Template'!$B$7</definedName>
     <definedName name="Table1_Player3_PairingPos" localSheetId="0">'Group Template'!$A$7</definedName>
     <definedName name="Table1_Player3_Quota" localSheetId="0">'Group Template'!$C$7</definedName>
+    <definedName name="Table1_Player3_TeeSetName" localSheetId="0">'Group Template'!$C$27</definedName>
     <definedName name="Table1_Player4_DisplayName" localSheetId="0">'Group Template'!$B$9</definedName>
     <definedName name="Table1_Player4_PairingPos" localSheetId="0">'Group Template'!$A$9</definedName>
     <definedName name="Table1_Player4_Quota" localSheetId="0">'Group Template'!$C$9</definedName>
+    <definedName name="Table1_Player4_TeeSetName" localSheetId="0">'Group Template'!$C$28</definedName>
     <definedName name="Table2" localSheetId="0">'Group Template'!$A$13:$Q$22</definedName>
     <definedName name="Table2_Hole01" localSheetId="0">'Group Template'!$E$13</definedName>
     <definedName name="Table2_Hole02" localSheetId="0">'Group Template'!$F$13</definedName>
@@ -81,7 +85,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="24">
   <si>
     <t>Pos</t>
   </si>
@@ -150,6 +154,9 @@
   </si>
   <si>
     <t>Group:</t>
+  </si>
+  <si>
+    <t>TEESET NAME</t>
   </si>
 </sst>
 </file>
@@ -167,17 +174,20 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="8"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="14"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
@@ -256,7 +266,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="32">
+  <borders count="25">
     <border>
       <left/>
       <right/>
@@ -315,6 +325,21 @@
         <color indexed="64"/>
       </right>
       <top/>
+      <bottom style="double">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
@@ -327,20 +352,37 @@
       <right style="thin">
         <color indexed="64"/>
       </right>
-      <top/>
-      <bottom style="double">
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="medium">
         <color indexed="64"/>
       </left>
       <right style="thin">
         <color indexed="64"/>
       </right>
-      <top style="medium">
+      <top style="thin">
         <color indexed="64"/>
       </top>
       <bottom style="thin">
@@ -352,13 +394,28 @@
       <left style="thin">
         <color indexed="64"/>
       </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
       <right style="thin">
         <color indexed="64"/>
       </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -367,13 +424,28 @@
       <left style="thin">
         <color indexed="64"/>
       </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
       <right style="medium">
         <color indexed="64"/>
       </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -388,9 +460,7 @@
       <top style="thin">
         <color indexed="64"/>
       </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
+      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -403,158 +473,7 @@
       <top style="thin">
         <color indexed="64"/>
       </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="double">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -687,7 +606,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -725,125 +644,146 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="16" fontId="5" fillId="5" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="16" fontId="5" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1026,7 +966,7 @@
         <v>22</v>
       </c>
       <c r="B1" s="1"/>
-      <c r="C1" s="44" t="s">
+      <c r="C1" s="22" t="s">
         <v>21</v>
       </c>
       <c r="D1" s="1"/>
@@ -1067,9 +1007,9 @@
       </c>
     </row>
     <row r="3" spans="1:17" s="4" customFormat="1" ht="25.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="42"/>
-      <c r="B3" s="40"/>
-      <c r="C3" s="40"/>
+      <c r="A3" s="31"/>
+      <c r="B3" s="33"/>
+      <c r="C3" s="33"/>
       <c r="D3" s="5" t="s">
         <v>6</v>
       </c>
@@ -1084,13 +1024,13 @@
       <c r="M3" s="6"/>
       <c r="N3" s="6"/>
       <c r="O3" s="7"/>
-      <c r="P3" s="45"/>
-      <c r="Q3" s="46"/>
+      <c r="P3" s="25"/>
+      <c r="Q3" s="28"/>
     </row>
     <row r="4" spans="1:17" s="4" customFormat="1" ht="25.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="43"/>
-      <c r="B4" s="41"/>
-      <c r="C4" s="41"/>
+      <c r="A4" s="32"/>
+      <c r="B4" s="34"/>
+      <c r="C4" s="34"/>
       <c r="D4" s="8" t="s">
         <v>5</v>
       </c>
@@ -1105,13 +1045,13 @@
       <c r="M4" s="9"/>
       <c r="N4" s="10"/>
       <c r="O4" s="9"/>
-      <c r="P4" s="47"/>
-      <c r="Q4" s="48"/>
+      <c r="P4" s="26"/>
+      <c r="Q4" s="29"/>
     </row>
     <row r="5" spans="1:17" s="4" customFormat="1" ht="25.8" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="42"/>
-      <c r="B5" s="40"/>
-      <c r="C5" s="40"/>
+      <c r="A5" s="31"/>
+      <c r="B5" s="33"/>
+      <c r="C5" s="33"/>
       <c r="D5" s="5" t="s">
         <v>6</v>
       </c>
@@ -1126,13 +1066,13 @@
       <c r="M5" s="6"/>
       <c r="N5" s="6"/>
       <c r="O5" s="7"/>
-      <c r="P5" s="47"/>
-      <c r="Q5" s="48"/>
+      <c r="P5" s="26"/>
+      <c r="Q5" s="29"/>
     </row>
     <row r="6" spans="1:17" s="4" customFormat="1" ht="25.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="43"/>
-      <c r="B6" s="41"/>
-      <c r="C6" s="41"/>
+      <c r="A6" s="32"/>
+      <c r="B6" s="34"/>
+      <c r="C6" s="34"/>
       <c r="D6" s="8" t="s">
         <v>5</v>
       </c>
@@ -1147,13 +1087,13 @@
       <c r="M6" s="9"/>
       <c r="N6" s="10"/>
       <c r="O6" s="9"/>
-      <c r="P6" s="47"/>
-      <c r="Q6" s="48"/>
+      <c r="P6" s="26"/>
+      <c r="Q6" s="29"/>
     </row>
     <row r="7" spans="1:17" s="4" customFormat="1" ht="25.8" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="42"/>
-      <c r="B7" s="40"/>
-      <c r="C7" s="40"/>
+      <c r="A7" s="31"/>
+      <c r="B7" s="33"/>
+      <c r="C7" s="33"/>
       <c r="D7" s="5" t="s">
         <v>6</v>
       </c>
@@ -1168,13 +1108,13 @@
       <c r="M7" s="6"/>
       <c r="N7" s="6"/>
       <c r="O7" s="7"/>
-      <c r="P7" s="47"/>
-      <c r="Q7" s="48"/>
+      <c r="P7" s="26"/>
+      <c r="Q7" s="29"/>
     </row>
     <row r="8" spans="1:17" s="4" customFormat="1" ht="25.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="43"/>
-      <c r="B8" s="41"/>
-      <c r="C8" s="41"/>
+      <c r="A8" s="32"/>
+      <c r="B8" s="34"/>
+      <c r="C8" s="34"/>
       <c r="D8" s="8" t="s">
         <v>5</v>
       </c>
@@ -1189,13 +1129,13 @@
       <c r="M8" s="9"/>
       <c r="N8" s="10"/>
       <c r="O8" s="9"/>
-      <c r="P8" s="47"/>
-      <c r="Q8" s="48"/>
+      <c r="P8" s="26"/>
+      <c r="Q8" s="29"/>
     </row>
     <row r="9" spans="1:17" s="4" customFormat="1" ht="25.8" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="42"/>
-      <c r="B9" s="40"/>
-      <c r="C9" s="40"/>
+      <c r="A9" s="31"/>
+      <c r="B9" s="33"/>
+      <c r="C9" s="33"/>
       <c r="D9" s="5" t="s">
         <v>6</v>
       </c>
@@ -1210,13 +1150,13 @@
       <c r="M9" s="6"/>
       <c r="N9" s="6"/>
       <c r="O9" s="7"/>
-      <c r="P9" s="47"/>
-      <c r="Q9" s="48"/>
+      <c r="P9" s="26"/>
+      <c r="Q9" s="29"/>
     </row>
     <row r="10" spans="1:17" s="4" customFormat="1" ht="25.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="43"/>
-      <c r="B10" s="41"/>
-      <c r="C10" s="41"/>
+      <c r="A10" s="32"/>
+      <c r="B10" s="34"/>
+      <c r="C10" s="34"/>
       <c r="D10" s="8" t="s">
         <v>5</v>
       </c>
@@ -1231,16 +1171,16 @@
       <c r="M10" s="9"/>
       <c r="N10" s="10"/>
       <c r="O10" s="9"/>
-      <c r="P10" s="49"/>
-      <c r="Q10" s="50"/>
+      <c r="P10" s="27"/>
+      <c r="Q10" s="30"/>
     </row>
     <row r="11" spans="1:17" s="4" customFormat="1" ht="25.8" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="39" t="s">
+      <c r="A11" s="35" t="s">
         <v>7</v>
       </c>
-      <c r="B11" s="39"/>
-      <c r="C11" s="39"/>
-      <c r="D11" s="39"/>
+      <c r="B11" s="35"/>
+      <c r="C11" s="35"/>
+      <c r="D11" s="35"/>
       <c r="E11" s="6"/>
       <c r="F11" s="6"/>
       <c r="G11" s="6"/>
@@ -1252,11 +1192,11 @@
       <c r="M11" s="6"/>
       <c r="N11" s="6"/>
       <c r="O11" s="6"/>
-      <c r="P11" s="51">
-        <f>QUOTIENT(C29,2)</f>
+      <c r="P11" s="23">
+        <f>QUOTIENT(E29,2)</f>
         <v>0</v>
       </c>
-      <c r="Q11" s="52"/>
+      <c r="Q11" s="24"/>
     </row>
     <row r="12" spans="1:17" s="4" customFormat="1" ht="7.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="11"/>
@@ -1313,9 +1253,9 @@
       </c>
     </row>
     <row r="14" spans="1:17" s="4" customFormat="1" ht="25.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="42"/>
-      <c r="B14" s="40"/>
-      <c r="C14" s="40"/>
+      <c r="A14" s="31"/>
+      <c r="B14" s="33"/>
+      <c r="C14" s="33"/>
       <c r="D14" s="5" t="s">
         <v>6</v>
       </c>
@@ -1330,13 +1270,13 @@
       <c r="M14" s="6"/>
       <c r="N14" s="6"/>
       <c r="O14" s="7"/>
-      <c r="P14" s="45"/>
-      <c r="Q14" s="46"/>
+      <c r="P14" s="25"/>
+      <c r="Q14" s="28"/>
     </row>
     <row r="15" spans="1:17" s="4" customFormat="1" ht="25.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="43"/>
-      <c r="B15" s="41"/>
-      <c r="C15" s="41"/>
+      <c r="A15" s="32"/>
+      <c r="B15" s="34"/>
+      <c r="C15" s="34"/>
       <c r="D15" s="8" t="s">
         <v>5</v>
       </c>
@@ -1351,13 +1291,13 @@
       <c r="M15" s="9"/>
       <c r="N15" s="10"/>
       <c r="O15" s="9"/>
-      <c r="P15" s="47"/>
-      <c r="Q15" s="48"/>
+      <c r="P15" s="26"/>
+      <c r="Q15" s="29"/>
     </row>
     <row r="16" spans="1:17" s="4" customFormat="1" ht="25.8" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="42"/>
-      <c r="B16" s="40"/>
-      <c r="C16" s="40"/>
+      <c r="A16" s="31"/>
+      <c r="B16" s="33"/>
+      <c r="C16" s="33"/>
       <c r="D16" s="5" t="s">
         <v>6</v>
       </c>
@@ -1372,13 +1312,13 @@
       <c r="M16" s="6"/>
       <c r="N16" s="6"/>
       <c r="O16" s="7"/>
-      <c r="P16" s="47"/>
-      <c r="Q16" s="48"/>
+      <c r="P16" s="26"/>
+      <c r="Q16" s="29"/>
     </row>
     <row r="17" spans="1:17" s="4" customFormat="1" ht="25.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="43"/>
-      <c r="B17" s="41"/>
-      <c r="C17" s="41"/>
+      <c r="A17" s="32"/>
+      <c r="B17" s="34"/>
+      <c r="C17" s="34"/>
       <c r="D17" s="8" t="s">
         <v>5</v>
       </c>
@@ -1393,13 +1333,13 @@
       <c r="M17" s="9"/>
       <c r="N17" s="10"/>
       <c r="O17" s="9"/>
-      <c r="P17" s="47"/>
-      <c r="Q17" s="48"/>
+      <c r="P17" s="26"/>
+      <c r="Q17" s="29"/>
     </row>
     <row r="18" spans="1:17" s="4" customFormat="1" ht="25.8" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="42"/>
-      <c r="B18" s="40"/>
-      <c r="C18" s="40"/>
+      <c r="A18" s="31"/>
+      <c r="B18" s="33"/>
+      <c r="C18" s="33"/>
       <c r="D18" s="5" t="s">
         <v>6</v>
       </c>
@@ -1414,13 +1354,13 @@
       <c r="M18" s="6"/>
       <c r="N18" s="6"/>
       <c r="O18" s="7"/>
-      <c r="P18" s="47"/>
-      <c r="Q18" s="48"/>
+      <c r="P18" s="26"/>
+      <c r="Q18" s="29"/>
     </row>
     <row r="19" spans="1:17" s="4" customFormat="1" ht="25.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="43"/>
-      <c r="B19" s="41"/>
-      <c r="C19" s="41"/>
+      <c r="A19" s="32"/>
+      <c r="B19" s="34"/>
+      <c r="C19" s="34"/>
       <c r="D19" s="8" t="s">
         <v>5</v>
       </c>
@@ -1435,13 +1375,13 @@
       <c r="M19" s="9"/>
       <c r="N19" s="10"/>
       <c r="O19" s="9"/>
-      <c r="P19" s="47"/>
-      <c r="Q19" s="48"/>
+      <c r="P19" s="26"/>
+      <c r="Q19" s="29"/>
     </row>
     <row r="20" spans="1:17" s="4" customFormat="1" ht="25.8" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="42"/>
-      <c r="B20" s="40"/>
-      <c r="C20" s="40"/>
+      <c r="A20" s="31"/>
+      <c r="B20" s="33"/>
+      <c r="C20" s="33"/>
       <c r="D20" s="5" t="s">
         <v>6</v>
       </c>
@@ -1456,13 +1396,13 @@
       <c r="M20" s="6"/>
       <c r="N20" s="6"/>
       <c r="O20" s="7"/>
-      <c r="P20" s="47"/>
-      <c r="Q20" s="48"/>
+      <c r="P20" s="26"/>
+      <c r="Q20" s="29"/>
     </row>
     <row r="21" spans="1:17" s="4" customFormat="1" ht="25.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="43"/>
-      <c r="B21" s="41"/>
-      <c r="C21" s="41"/>
+      <c r="A21" s="32"/>
+      <c r="B21" s="34"/>
+      <c r="C21" s="34"/>
       <c r="D21" s="8" t="s">
         <v>5</v>
       </c>
@@ -1477,16 +1417,16 @@
       <c r="M21" s="9"/>
       <c r="N21" s="10"/>
       <c r="O21" s="9"/>
-      <c r="P21" s="49"/>
-      <c r="Q21" s="50"/>
+      <c r="P21" s="27"/>
+      <c r="Q21" s="30"/>
     </row>
     <row r="22" spans="1:17" s="4" customFormat="1" ht="25.8" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="39" t="s">
+      <c r="A22" s="35" t="s">
         <v>7</v>
       </c>
-      <c r="B22" s="39"/>
-      <c r="C22" s="39"/>
-      <c r="D22" s="39"/>
+      <c r="B22" s="35"/>
+      <c r="C22" s="35"/>
+      <c r="D22" s="35"/>
       <c r="E22" s="6"/>
       <c r="F22" s="6"/>
       <c r="G22" s="6"/>
@@ -1498,153 +1438,202 @@
       <c r="M22" s="6"/>
       <c r="N22" s="6"/>
       <c r="O22" s="6"/>
-      <c r="P22" s="51">
-        <f>QUOTIENT(C29,2)+IF(MOD(C29,2)=1,1,0)</f>
+      <c r="P22" s="23">
+        <f>QUOTIENT(E29,2)+IF(MOD(E29,2)=1,1,0)</f>
         <v>0</v>
       </c>
-      <c r="Q22" s="52"/>
+      <c r="Q22" s="24"/>
     </row>
     <row r="23" spans="1:17" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="24" spans="1:17" s="4" customFormat="1" ht="20.399999999999999" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="35" t="s">
+    <row r="24" spans="1:17" s="4" customFormat="1" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="40" t="s">
         <v>8</v>
       </c>
-      <c r="B24" s="36"/>
-      <c r="C24" s="15" t="s">
+      <c r="B24" s="41"/>
+      <c r="C24" s="56" t="s">
+        <v>23</v>
+      </c>
+      <c r="D24" s="57"/>
+      <c r="E24" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="F24" s="26" t="s">
+      <c r="H24" s="44" t="s">
         <v>19</v>
       </c>
-      <c r="G24" s="27" t="s">
+      <c r="I24" s="45" t="s">
         <v>20</v>
       </c>
-      <c r="H24" s="28" t="s">
+      <c r="J24" s="46" t="s">
         <v>17</v>
       </c>
-      <c r="O24" s="35" t="s">
+      <c r="O24" s="40" t="s">
         <v>10</v>
       </c>
-      <c r="P24" s="36"/>
+      <c r="P24" s="41"/>
       <c r="Q24" s="15" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="25" spans="1:17" s="4" customFormat="1" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="37">
+      <c r="A25" s="42">
         <f>B3</f>
         <v>0</v>
       </c>
-      <c r="B25" s="38"/>
-      <c r="C25" s="13">
+      <c r="B25" s="43"/>
+      <c r="C25" s="58"/>
+      <c r="D25" s="58"/>
+      <c r="E25" s="13">
         <f>C3</f>
         <v>0</v>
       </c>
-      <c r="F25" s="23"/>
-      <c r="G25" s="24"/>
-      <c r="H25" s="25"/>
-      <c r="O25" s="29" t="s">
+      <c r="H25" s="47"/>
+      <c r="I25" s="21"/>
+      <c r="J25" s="13"/>
+      <c r="O25" s="36" t="s">
         <v>11</v>
       </c>
-      <c r="P25" s="30"/>
+      <c r="P25" s="37"/>
       <c r="Q25" s="13">
         <v>6</v>
       </c>
     </row>
     <row r="26" spans="1:17" s="4" customFormat="1" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="37">
+      <c r="A26" s="42">
         <f>B5</f>
         <v>0</v>
       </c>
-      <c r="B26" s="38"/>
-      <c r="C26" s="13">
+      <c r="B26" s="43"/>
+      <c r="C26" s="58"/>
+      <c r="D26" s="58"/>
+      <c r="E26" s="13">
         <f>C5</f>
         <v>0</v>
       </c>
-      <c r="F26" s="16"/>
-      <c r="G26" s="12"/>
-      <c r="H26" s="17"/>
-      <c r="O26" s="29" t="s">
+      <c r="H26" s="16"/>
+      <c r="I26" s="12"/>
+      <c r="J26" s="17"/>
+      <c r="O26" s="36" t="s">
         <v>12</v>
       </c>
-      <c r="P26" s="30"/>
+      <c r="P26" s="37"/>
       <c r="Q26" s="13">
         <v>4</v>
       </c>
     </row>
     <row r="27" spans="1:17" s="4" customFormat="1" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="37">
+      <c r="A27" s="42">
         <f>B7</f>
         <v>0</v>
       </c>
-      <c r="B27" s="38"/>
-      <c r="C27" s="13">
+      <c r="B27" s="43"/>
+      <c r="C27" s="58"/>
+      <c r="D27" s="58"/>
+      <c r="E27" s="13">
         <f>C7</f>
         <v>0</v>
       </c>
-      <c r="F27" s="16"/>
-      <c r="G27" s="12"/>
-      <c r="H27" s="17"/>
-      <c r="O27" s="29" t="s">
+      <c r="H27" s="16"/>
+      <c r="I27" s="12"/>
+      <c r="J27" s="17"/>
+      <c r="O27" s="36" t="s">
         <v>13</v>
       </c>
-      <c r="P27" s="30"/>
+      <c r="P27" s="37"/>
       <c r="Q27" s="13">
         <v>2</v>
       </c>
     </row>
     <row r="28" spans="1:17" s="4" customFormat="1" ht="20.399999999999999" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A28" s="37">
+      <c r="A28" s="51">
         <f>B9</f>
         <v>0</v>
       </c>
-      <c r="B28" s="38"/>
-      <c r="C28" s="14">
+      <c r="B28" s="52"/>
+      <c r="C28" s="59"/>
+      <c r="D28" s="59"/>
+      <c r="E28" s="53">
         <f>C9</f>
         <v>0</v>
       </c>
-      <c r="F28" s="18"/>
-      <c r="G28" s="19"/>
-      <c r="H28" s="20"/>
-      <c r="O28" s="29" t="s">
+      <c r="H28" s="18"/>
+      <c r="I28" s="19"/>
+      <c r="J28" s="20"/>
+      <c r="O28" s="36" t="s">
         <v>14</v>
       </c>
-      <c r="P28" s="30"/>
+      <c r="P28" s="37"/>
       <c r="Q28" s="13">
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:17" s="4" customFormat="1" ht="20.399999999999999" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="33" t="s">
+    <row r="29" spans="1:17" s="4" customFormat="1" ht="20.399999999999999" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A29" s="54" t="s">
         <v>18</v>
       </c>
-      <c r="B29" s="34"/>
-      <c r="C29" s="21">
-        <f>SUM(C25:C28)</f>
+      <c r="B29" s="55"/>
+      <c r="C29" s="55" t="s">
+        <v>18</v>
+      </c>
+      <c r="D29" s="55"/>
+      <c r="E29" s="50">
+        <f>SUM(E25:E28)</f>
         <v>0</v>
       </c>
-      <c r="F29" s="22"/>
-      <c r="G29" s="22"/>
-      <c r="H29" s="22"/>
-      <c r="O29" s="29" t="s">
+      <c r="H29" s="48"/>
+      <c r="I29" s="49"/>
+      <c r="J29" s="50"/>
+      <c r="O29" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="P29" s="30"/>
+      <c r="P29" s="37"/>
       <c r="Q29" s="13">
         <v>0</v>
       </c>
     </row>
     <row r="30" spans="1:17" s="4" customFormat="1" ht="20.399999999999999" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="O30" s="31" t="s">
+      <c r="O30" s="38" t="s">
         <v>16</v>
       </c>
-      <c r="P30" s="32"/>
+      <c r="P30" s="39"/>
       <c r="Q30" s="14">
         <v>-1</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="43">
+  <mergeCells count="49">
+    <mergeCell ref="C27:D27"/>
+    <mergeCell ref="C28:D28"/>
+    <mergeCell ref="C29:D29"/>
+    <mergeCell ref="O29:P29"/>
+    <mergeCell ref="O30:P30"/>
+    <mergeCell ref="A29:B29"/>
+    <mergeCell ref="O24:P24"/>
+    <mergeCell ref="O25:P25"/>
+    <mergeCell ref="O26:P26"/>
+    <mergeCell ref="O27:P27"/>
+    <mergeCell ref="O28:P28"/>
+    <mergeCell ref="A25:B25"/>
+    <mergeCell ref="A26:B26"/>
+    <mergeCell ref="A27:B27"/>
+    <mergeCell ref="A28:B28"/>
+    <mergeCell ref="A24:B24"/>
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="A22:D22"/>
+    <mergeCell ref="C18:C19"/>
+    <mergeCell ref="C20:C21"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="A11:D11"/>
+    <mergeCell ref="C16:C17"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="A18:A19"/>
+    <mergeCell ref="B18:B19"/>
+    <mergeCell ref="A20:A21"/>
+    <mergeCell ref="B20:B21"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="C14:C15"/>
     <mergeCell ref="P3:P10"/>
     <mergeCell ref="Q3:Q10"/>
     <mergeCell ref="A14:A15"/>
@@ -1661,33 +1650,6 @@
     <mergeCell ref="C3:C4"/>
     <mergeCell ref="C5:C6"/>
     <mergeCell ref="C7:C8"/>
-    <mergeCell ref="A22:D22"/>
-    <mergeCell ref="C18:C19"/>
-    <mergeCell ref="C20:C21"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="B9:B10"/>
-    <mergeCell ref="A11:D11"/>
-    <mergeCell ref="C16:C17"/>
-    <mergeCell ref="B16:B17"/>
-    <mergeCell ref="A18:A19"/>
-    <mergeCell ref="B18:B19"/>
-    <mergeCell ref="A20:A21"/>
-    <mergeCell ref="B20:B21"/>
-    <mergeCell ref="C9:C10"/>
-    <mergeCell ref="C14:C15"/>
-    <mergeCell ref="O29:P29"/>
-    <mergeCell ref="O30:P30"/>
-    <mergeCell ref="A29:B29"/>
-    <mergeCell ref="O24:P24"/>
-    <mergeCell ref="O25:P25"/>
-    <mergeCell ref="O26:P26"/>
-    <mergeCell ref="O27:P27"/>
-    <mergeCell ref="O28:P28"/>
-    <mergeCell ref="A25:B25"/>
-    <mergeCell ref="A26:B26"/>
-    <mergeCell ref="A27:B27"/>
-    <mergeCell ref="A28:B28"/>
-    <mergeCell ref="A24:B24"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0.53" bottom="0.22" header="0.22" footer="0.18"/>

</xml_diff>